<commit_message>
Digest 2026-07-10 (recovered leftover run output)
</commit_message>
<xml_diff>
--- a/state/reading_log.xlsx
+++ b/state/reading_log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1986,7 +1986,6 @@
           <t>This study shows that serial-order effects in route learning combine additively with environmental-geometry effects on spatial memory, with the worst location memory occurring at the end of routes through the most irregular (trapezoid) environments. That additive combination of a position-in-sequence effect and an environment-shape effect is a useful precedent for the location-sequence version of the mouse task you're currently developing, where sequence elements are defined by spatial position rather than pitch: it suggests position-dependent memory effects (like the primacy bias you're probing in Protocol 8) and physical/geometric context could combine rather than trade off, which becomes testable once that task has enough conditions to separate the two factors.</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>No</t>
@@ -2009,7 +2008,6 @@
           <t>Neuronal dynamics, timing, and flow of sensory and choice-related information in auditory-prefrontal circuitry</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>Bruno B. Averbeck</t>
@@ -2050,7 +2048,6 @@
           <t>Recording from macaque auditory cortex and prefrontal cortex during an auditory decision task, this group shows that raw sensory information flows in the feedforward direction (auditory cortex to prefrontal cortex) while choice-related information flows bidirectionally between the two regions — a clean dissociation of what propagates forward versus what involves both areas jointly. This is close to a direct analogue of the mouse sequence-discrimination task's core question of how auditory cortex and prelimbic cortex jointly support the go/no-go decision: the directional/timing analysis here is a template for asking whether your own Neuropixels recordings from prelimbic and auditory cortex show the same feedforward-sensory/bidirectional-choice pattern around the decision window at the last chord.</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>No</t>
@@ -2118,7 +2115,6 @@
           <t>Using fiber photometry, single-cell calcium imaging, and optogenetic inhibition in mouse medial prefrontal cortex during learned avoidance tasks, this study finds that GABAergic medial-prefrontal neurons encode cues, actions, and outcomes with increasing task complexity, but silencing that cortex has minimal effect on learning or performance — its activity reflects movement and evaluative signals rather than causally generating the action. That's a direct methodological caution for the prelimbic-cortex recordings in the mouse sequence-discrimination task: a region can carry rich task-related information, which your prelimbic Neuropixels data will likely also show, without being causally necessary for the behavior, so any causal claim about prelimbic cortex driving the go/no-go decision would need its own inactivation experiment, not just encoding strength.</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>No</t>
@@ -2186,7 +2182,6 @@
           <t>Using laminar-resolution fMRI during a cascading auditory oddball paradigm, this study (co-authored by watch-listed predictive-processing researcher Ryszard Auksztulewicz) localizes prediction-error signals to superficial cortical layers of planum polare and middle layers of lateral temporal cortex, with model-updating tied to deep-layer activity — evidence for a layer-specific implementation of hierarchical predictive coding in human auditory cortex. This gives a concrete laminar target for the statistical-learning side of the human chunk-in-stream task: if high-gamma responses during the statistical-background-variation stage of that task (where bottom-up pattern extraction and top-down template matching are meant to dissociate) show a similar superficial-versus-deep split, that would support reading prediction-error and model-update signals off different cortical depths rather than treating high-gamma as one undifferentiated regularity signal.</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>No</t>
@@ -2254,7 +2249,6 @@
           <t>Recording over 18,000 neurons across 16 brain regions in young and aged mice performing a visual decision task, this group shows that aging increases post-stimulus neural variability (Fano factor) and reduces stimulus-induced variability quenching, with region-specific direction — higher firing in cortex and striatum, lower in thalamus. This is a large-scale demonstration of exactly the kind of continuous, state-dependent framing your GLM Module C (slow drift from satiety or time-on-task) is trying to capture in the mouse sequence-discrimination task: variability-quenching metrics like theirs could be applied session-by-session to your prelimbic and auditory cortex recordings to ask whether within-session drift in engagement shows up as a comparable loss of stimulus-locked variability reduction, independent of your existing hit/false-alarm-based Module C features.</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
           <t>No</t>
@@ -2322,7 +2316,6 @@
           <t>Using MEG during a visuomotor task with non-adjacent temporal dependencies embedded in noise, this study (with watch-listed statistical-learning researcher Dezső Németh as a co-author) dissociates two temporally separate learning mechanisms: a fast-emerging neural predictive-activity signal that appears before behavioral improvement, and a slower-building representational change that increases neural pattern similarity between the statistically dependent elements. This maps directly onto the bottom-up-statistical-learning-versus-top-down-template-matching framing at the core of the human chunk-in-stream task's design, and gives a concrete analysis template — pre-stimulus predictive decoding versus pattern-similarity growth across sessions — for separating those two processes in your own high-gamma and single-unit data as target sequences move toward full multi-template scene analysis.</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>No</t>
@@ -2390,7 +2383,6 @@
           <t>This preprint fits a Hierarchical Bayesian Statistical Learning model to individual EEG-derived learning trajectories as adults with and without dyslexia listen to structured tone sequences, and shows the model's simulated sequences closely match what participants actually generated — a working proof of concept for individual-level generative models of sequence learning. It's a useful methodological cousin to your own per-session model-fitting toolchain (the 24-model leaky-accumulator family fit by differential evolution, plus the tiered GLM strategy models): both try to recover an individual's latent learning process from sequence behavior, and this hierarchical Bayesian framing is worth comparing against your AICc/Akaike-weight model selection as an alternative way to handle per-mouse or per-session variability in the tone-sequence version of your task.</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>No</t>
@@ -2413,7 +2405,6 @@
           <t>Multi-network Topology Underlying Individual Language Learning Success</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>Gangyi Feng</t>
@@ -2454,7 +2445,6 @@
           <t>Using multimodal neuroimaging before and during seven days of artificial-language training across six tasks (auditory/speech categories, words, morphosyntax, sentence structure), this study finds that individual differences in learning outcome and rate are best predicted by the local efficiency of the dorsal-attention and frontoparietal control networks, not classic frontotemporal language regions alone. That distributed-network account of language-learning success is a relevant frame for the top-down template-matching side of the human chunk-in-stream task, particularly at the participant's frontoparietal recording sites (inferior and middle frontal gyrus): if attention/control-network engagement predicts how quickly a new stimulus class is learned, that argues for tracking frontoparietal signal quality across sessions when comparing performance across the harmonic-chord, vowel, and syllable stimulus classes.</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>No</t>
@@ -2497,7 +2487,6 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>2026</t>
@@ -2518,7 +2507,6 @@
           <t>In a closed-loop test with a participant implanted with bilateral intracortical microelectrode arrays, this group shows that ensembling multiple independently trained decoders reduces speech brain-computer-interface word-error rate from 33.7% to 26.0%, and introduces a cheaper pseudo-ensembling method (test-time augmentation on a single decoder) that captures much of the benefit without the full computational cost. This is directly relevant to the human chunk-in-stream work's broader translational context — intracortical decoding in a person with severe language impairment — and the pseudo-ensembling trick is a concretely reusable idea for your own single-unit and high-gamma decoding pipelines in angular gyrus, supramarginal gyrus, and frontal sites, where training data per session is similarly limited by session count.</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr">
         <is>
           <t>No</t>
@@ -2541,7 +2529,6 @@
           <t>KIASORT: Knowledge-Integrated Automated Spike Sorting for Geometry-Free Neuron Tracking</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>Kianoush Banaie Boroujeni</t>
@@ -2582,7 +2569,6 @@
           <t>KIASORT is a new geometry-free spike-sorting algorithm that tracks each neuron's waveform drift independently rather than assuming a shared one-dimensional drift model across the probe, and the authors show it outperforms Kilosort4 on ground-truth benchmarks with heterogeneous per-neuron drift, validated on both primate and mouse data. Since your mouse Neuropixels 2.0 recordings from prelimbic and auditory cortex are currently sorted with Kilosort and drift is a known problem for long recordings, this is a direct pipeline-upgrade candidate worth benchmarking against your existing output — particularly if you've noticed unit-identity or waveform instability across a session, which per-neuron drift tracking is specifically designed to fix.</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
           <t>No</t>
@@ -2650,7 +2636,6 @@
           <t>This paper introduces Neuropixels Opto, a probe integrating 960 recording sites with 28 independently addressable light emitters on the same shank, enabling spatially targeted optogenetic activation or silencing at specific cortical depths during high-density recording, and demonstrates efficient two-cell-type optotagging in mouse striatum. For the mouse sequence-discrimination task, where you already use Neuropixels 2.0 in prelimbic and auditory cortex, this would let you causally test which cortical layer or cell type carries the decision signal you currently only characterize correlationally — for instance, silencing superficial versus deep layers during the decision window to ask whether the prelimbic signal is more like the movement/evaluative activity described in today's medial-prefrontal-cortex threat paper, or a genuine causal driver of the go/no-go choice.</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr">
         <is>
           <t>No</t>
@@ -2718,7 +2703,6 @@
           <t>This preprint directly compares frequentist null-hypothesis testing against a Bayesian evidence-accumulation framework for adjudicating between competing computational models of an auditory processing pathway (loudness processing), arguing the Bayesian approach better handles collinear/competing models and yields a genuine measure of relative evidence rather than a simple reject/fail-to-reject decision. This is a close methodological parallel to your own model-selection practice — AICc and Akaike weights across your 24 nested drift-diffusion models, and cross-validated information gain for the GLM strategy models — and is worth reading as a check on whether a fully Bayesian evidence framework would handle collinearity between your structurally similar nested models (for instance leaky integration versus urgency) better than AICc currently does.</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
           <t>No</t>
@@ -2786,7 +2770,6 @@
           <t>This group shows, via a circuit model plus multi-area population recordings, that the dominant axis of shared trial-to-trial variability in sensory neurons consistently aligns with task-relevant stimulus features and action plans, and that this shared-variability axis predicts the behavioral effect of microstimulation — reframing correlated variability as something that reveals rather than obscures the information sent downstream. This is a useful population-analysis framing for your own auditory cortex and prelimbic Neuropixels data: rather than treating trial-to-trial variability purely as noise to average out in dPCA or mixed-selectivity analyses, it's worth checking whether the low-dimensional axis of shared variability in your target-chord-evoked responses aligns with the decision-relevant dimension your GLM Module A features already isolate.</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
           <t>No</t>
@@ -2854,13 +2837,344 @@
           <t>This group simultaneously recorded EEG and markerless-pose-estimation-based body kinematics from 79 infants (3, 6, and 12 months) listening to music, finding that enhanced neural auditory responses to music are present from 3 months, but structured, complex movement patterns in response to music only emerge by 12 months — auditory encoding and motor response to sound develop on different timescales. This sits squarely inside your standing interest in continuous, pose-estimation-based behavioral quantification rather than per-trial outcomes, and offers a conceptual mirror for the mouse work: it's a reminder that a subject can show clear neural sensitivity to a sound sequence's structure well before that sensitivity is expressed in structured movement — relevant when interpreting mice that discriminate the target sequence from its reordered distractor in evoked activity but haven't yet generalized that to a reliable licking response, especially under the currently-running slow-pacing protocol.</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Effect of tempo on newborns' neural processing of auditory rhythm: Emergence of sensitivity to metrical structure</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Edalati, M. et al.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Sahar Moghimi</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>University of Picardie Jules Verne</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>bioRxiv</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.07.07.736947</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Chunking &amp; sequence processing</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Newborns show neural sensitivity not just to a repeating auditory beat but to the slower beat-grouping periodicities (pairs or triples of beats forming a metrical hierarchy), and critically this hierarchical sensitivity only emerges at some tempi and not others, suggesting the immature auditory system has tempo-dependent limits on how much temporal structure it can extract at once. This is a direct developmental precedent for your own chord-sequence-in-stream work: your target sequence is itself a small hierarchy (a fixed 3-4 element chunk that must be detected regardless of surrounding context), and this paper's tempo-dependent breakdown of grouping sensitivity is a concrete reason to ask whether your own chord duration and inter-chord interval (150 ms/150 ms) sit inside or outside the window where a naive listener (or a mouse early in training) could extract hierarchical structure at all before learning kicks in.</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Medial prefrontal cortex encodes but is not required to generate goal-directed actions under threat.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Muhammad S Sajid et al.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Manuel A. Castro-Alamancos</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>University of Connecticut</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>eLife</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/42417528/</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Auditory &amp; prefrontal electrophysiology</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Using fiber photometry, single-cell calcium imaging, and optogenetic inhibition in mouse medial prefrontal cortex during a learned avoidance task, the authors show that a large share of apparent task-related activity in this region is actually shared with a control, non-task cortical area once movement and arousal are properly regressed out, and that silencing the mPFC GABAergic neurons with the cleanest encoding of demanding avoidance contingencies had almost no effect on learning or performance. This is a direct methodological caution for your prelimbic cortex recordings during the mouse sequence-discrimination task: it argues for validating any decision-window encoding you find in prelimbic cortex against a control region and, where possible, an optogenetic perturbation, before treating anticipatory discrimination signals as causally load-bearing rather than a correlate of behavioral state.</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>A corticostriatal circuit updates subjective beliefs about latent task states</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Margaret L. DeMaegd et al.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Christine M. Constantinople</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>New York University</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.03.12.711369</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Behavioral &amp; computational modeling</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Projection-specific recordings and optogenetic perturbations from orbitofrontal neurons projecting to the caudoputamen in rats performing a hidden-reward-state task show that this corticostriatal pathway encodes categorical evidence for a latent state and that downstream neurons could in principle decode the animal's full belief distribution over states as it deliberates, giving a circuit-level implementation of belief updating about an abstract, non-observable variable. This is the closest circuit-level precedent I've seen for what your own GLM Module C (slow drifts in strategy from satiety or time-on-task) is trying to capture behaviorally: it suggests a concrete corticostriatal locus you could look to, or at least borrow the belief-decoding logic from, if you ever want to move Module C from a behavioral drift term into a claim about what a specific circuit is representing.</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Visual working memory guides attention rhythmically in humans.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Jiachen Lu et al.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Xilin Zhang</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>South China Normal University</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>eLife</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/42418336/</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Circuits, methods &amp; population analysis</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Rather than one or many working-memory items being simultaneously available as an attentional template, this paper finds that two remembered items alternately dominate behavioral guidance at a theta rhythm (4-8 Hz), with frontal theta phase leading the occipital alpha oscillation that tracks which item is currently prioritized. If template-guided attention is intrinsically rhythmic rather than continuously available, it's worth asking whether hit/miss timing in your human chunk-in-stream detection task shows periodicity locked to either the stimulus tempo or an endogenous rhythm, which would suggest the memorized target template is only intermittently 'online' for comparison against the incoming stream rather than being a static comparison signal.</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>C1q and immunoglobulins mediate activity-dependent synapse loss in the adult brain</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Beth Stevens</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Harvard Medical School</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/abs/10.1126/science.adv1219?af=R</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Other notable</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>This Science paper (with an accompanying perspective piece, 'Antibodies sculpt adult brain circuits') shows that neuronal hyperactivity triggers region-specific deposition of complement protein C1q, and that B-lymphocyte-lineage cells and immunoglobulins are required for this activity-dependent synapse elimination in the adult hippocampus, extending complement-mediated pruning (previously known mainly from development and disease) into ongoing, activity-driven circuit refinement in the healthy adult brain. It sits well outside your auditory/sequence paradigm, but it is a field-defining mechanistic result about how immune signaling gates activity-dependent circuit remodeling, which is the same general class of question (what determines which synapses survive experience-driven plasticity) that sits underneath the auditory-cortex critical-period literature already in your canon list.</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>